<commit_message>
Update header with company, film title and project name
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013sgCJY4DwRWjuY7qnd4uaw
</commit_message>
<xml_diff>
--- a/TIFF行程预算.xlsx
+++ b/TIFF行程预算.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="56">
   <si>
     <r>
       <rPr>
@@ -43,6 +43,33 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">廿一影视</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">片名</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">:</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Beans and Belief</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b val="true"/>
@@ -64,23 +91,7 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">黑豆 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(Black Bean)</t>
-    </r>
+    <t xml:space="preserve">TIFF</t>
   </si>
   <si>
     <r>
@@ -379,72 +390,13 @@
     <t xml:space="preserve">1000</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">机票 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">FLIGHTS</t>
-    </r>
+    <t xml:space="preserve">机票 FLIGHTS</t>
   </si>
   <si>
     <t xml:space="preserve">100101</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">机票 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">色珍 — 拉萨</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">北京</t>
-    </r>
+    <t xml:space="preserve">机票 / 色珍 — 拉萨-北京</t>
   </si>
   <si>
     <t xml:space="preserve">电影节</t>
@@ -459,117 +411,19 @@
     <t xml:space="preserve">100102</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">机票 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">色珍 — 北京</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">多伦多</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">拉萨</t>
-    </r>
+    <t xml:space="preserve">机票 / 色珍 — 北京-多伦多-拉萨</t>
   </si>
   <si>
     <t xml:space="preserve">往返</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">往返；色珍机票合计 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">20,200</t>
-    </r>
+    <t xml:space="preserve">往返；色珍机票合计 20,200</t>
   </si>
   <si>
     <t xml:space="preserve">100103</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">机票 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">水素 — 往返</t>
-    </r>
+    <t xml:space="preserve">机票 / 水素 — 往返</t>
   </si>
   <si>
     <t xml:space="preserve">水素</t>
@@ -578,94 +432,13 @@
     <t xml:space="preserve">2000</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">住宿 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">ACCOMMODATION</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">（</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Airbnb</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">，</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">USD</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">计价）</t>
-    </r>
+    <t xml:space="preserve">住宿 ACCOMMODATION（Airbnb，USD计价）</t>
   </si>
   <si>
     <t xml:space="preserve">200101</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">住宿 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ Airbnb</t>
-    </r>
+    <t xml:space="preserve">住宿 / Airbnb</t>
   </si>
   <si>
     <r>
@@ -805,100 +578,13 @@
     <t xml:space="preserve">3000</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">餐饮 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">FOOD &amp; PER DIEM</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">（</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">USD</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">计价）</t>
-    </r>
+    <t xml:space="preserve">餐饮 FOOD &amp; PER DIEM（USD计价）</t>
   </si>
   <si>
     <t xml:space="preserve">300101</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">餐饮 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ Per Diem — 1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">人</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">×14</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">天</t>
-    </r>
+    <t xml:space="preserve">餐饮 / Per Diem — 1人×14天</t>
   </si>
   <si>
     <r>
@@ -995,22 +681,17 @@
     <t xml:space="preserve">300102</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">餐饮 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ Per Diem — 1</t>
+    <t xml:space="preserve">餐饮 / Per Diem — 1人×8天</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">$50/</t>
     </r>
     <r>
       <rPr>
@@ -1027,26 +708,41 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">×8</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">天</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">$50/</t>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">天 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">× 8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">天 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">× 1</t>
     </r>
     <r>
       <rPr>
@@ -1056,104 +752,15 @@
       </rPr>
       <t xml:space="preserve">人</t>
     </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">天 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">× 8</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">天 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">× 1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">人</t>
-    </r>
   </si>
   <si>
     <t xml:space="preserve">4000</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">不可预见费 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">CONTINGENCY</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">总计 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">GRAND TOTAL</t>
-    </r>
+    <t xml:space="preserve">不可预见费 CONTINGENCY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">总计 GRAND TOTAL</t>
   </si>
 </sst>
 </file>
@@ -1166,7 +773,7 @@
     <numFmt numFmtId="166" formatCode="#,##0.00"/>
     <numFmt numFmtId="167" formatCode="0.00%"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1204,19 +811,26 @@
     </font>
     <font>
       <sz val="9"/>
-      <color rgb="FF0000FF"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="WenQuanYi Zen Hei"/>
-      <family val="2"/>
+      <name val="Noto Sans CJK SC"/>
+      <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
       <sz val="9"/>
-      <name val="Noto Sans CJK SC"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -1228,7 +842,21 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
       <sz val="9"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1238,14 +866,13 @@
       <color rgb="FF0000FF"/>
       <name val="WenQuanYi Zen Hei"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
       <sz val="9"/>
       <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -1261,6 +888,7 @@
       <color rgb="FFFFFFFF"/>
       <name val="WenQuanYi Zen Hei"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -1357,84 +985,92 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1442,43 +1078,43 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="16" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="16" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1737,435 +1373,443 @@
   <dimension ref="A1:K22"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="46"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>2</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="4" t="s">
+      <c r="A3" s="2" t="s">
         <v>4</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="4" t="s">
+      <c r="A4" s="2" t="s">
         <v>6</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="2" t="s">
+      <c r="A5" s="2" t="s">
         <v>8</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="5" t="n">
+      <c r="A6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="7" t="n">
         <v>6.73</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="6" t="s">
+      <c r="A7" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="B7" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="C7" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="D7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="E7" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="F7" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="J7" s="7" t="s">
+      <c r="G7" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="K7" s="7" t="s">
+      <c r="H7" s="8" t="s">
         <v>20</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="J7" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="K7" s="9" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="10" t="n">
+      <c r="A8" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="12" t="n">
         <f aca="false">SUM(I9:I11)</f>
         <v>32200</v>
       </c>
-      <c r="J8" s="11" t="n">
+      <c r="J8" s="13" t="n">
         <f aca="false">IF(OR($I8="",$I$22=0),"",$I8/$I$22)</f>
         <v>0.439743528463834</v>
       </c>
-      <c r="K8" s="9"/>
+      <c r="K8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="B9" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="D9" s="14" t="s">
+      <c r="A9" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="B9" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="E9" s="17" t="n">
         <v>2200</v>
       </c>
-      <c r="F9" s="16" t="n">
+      <c r="F9" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="H9" s="16" t="n">
+      <c r="G9" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="H9" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="I9" s="18" t="n">
+      <c r="I9" s="20" t="n">
         <f aca="false">IF($E9="","",$E9*IF($F9="",1,$F9)*IF($H9="",1,$H9))</f>
         <v>2200</v>
       </c>
-      <c r="J9" s="19" t="n">
+      <c r="J9" s="21" t="n">
         <f aca="false">IF(OR($I9="",$I$22=0),"",$I9/$I$22)</f>
         <v>0.0300445889012557</v>
       </c>
-      <c r="K9" s="13" t="s">
-        <v>27</v>
+      <c r="K9" s="15" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="D10" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" s="15" t="n">
+      <c r="E10" s="17" t="n">
         <v>18000</v>
       </c>
-      <c r="F10" s="16" t="n">
+      <c r="F10" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="H10" s="16" t="n">
+      <c r="G10" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="H10" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="I10" s="18" t="n">
+      <c r="I10" s="20" t="n">
         <f aca="false">IF($E10="","",$E10*IF($F10="",1,$F10)*IF($H10="",1,$H10))</f>
         <v>18000</v>
       </c>
-      <c r="J10" s="19" t="n">
+      <c r="J10" s="21" t="n">
         <f aca="false">IF(OR($I10="",$I$22=0),"",$I10/$I$22)</f>
         <v>0.245819363737547</v>
       </c>
-      <c r="K10" s="13" t="s">
-        <v>31</v>
+      <c r="K10" s="15" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="13" t="s">
+      <c r="A11" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="E11" s="17" t="n">
+        <v>12000</v>
+      </c>
+      <c r="F11" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="D11" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="E11" s="15" t="n">
-        <v>12000</v>
-      </c>
-      <c r="F11" s="16" t="n">
+      <c r="H11" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="H11" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" s="18" t="n">
+      <c r="I11" s="20" t="n">
         <f aca="false">IF($E11="","",$E11*IF($F11="",1,$F11)*IF($H11="",1,$H11))</f>
         <v>12000</v>
       </c>
-      <c r="J11" s="19" t="n">
+      <c r="J11" s="21" t="n">
         <f aca="false">IF(OR($I11="",$I$22=0),"",$I11/$I$22)</f>
         <v>0.163879575825031</v>
       </c>
-      <c r="K11" s="13" t="s">
-        <v>30</v>
+      <c r="K11" s="15" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="10" t="n">
+      <c r="A13" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="12" t="n">
         <f aca="false">SUM(I14:I14)</f>
         <v>30621.5</v>
       </c>
-      <c r="J13" s="11" t="n">
+      <c r="J13" s="13" t="n">
         <f aca="false">IF(OR($I13="",$I$22=0),"",$I13/$I$22)</f>
         <v>0.418186535927183</v>
       </c>
-      <c r="K13" s="9"/>
+      <c r="K13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="D14" s="14"/>
-      <c r="E14" s="15" t="n">
+      <c r="A14" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" s="16"/>
+      <c r="E14" s="17" t="n">
         <v>350</v>
       </c>
-      <c r="F14" s="16" t="n">
+      <c r="F14" s="18" t="n">
         <v>13</v>
       </c>
-      <c r="G14" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="H14" s="16" t="n">
+      <c r="G14" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="H14" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="I14" s="18" t="n">
-        <f aca="false">IF($E14="","",$E14*$B$6*IF($F14="",1,$F14)*IF($H14="",1,$H14))</f>
+      <c r="I14" s="20" t="n">
+        <f aca="false">IF($E14="","",$E14*$E$6*IF($F14="",1,$F14)*IF($H14="",1,$H14))</f>
         <v>30621.5</v>
       </c>
-      <c r="J14" s="19" t="n">
+      <c r="J14" s="21" t="n">
         <f aca="false">IF(OR($I14="",$I$22=0),"",$I14/$I$22)</f>
         <v>0.418186535927183</v>
       </c>
-      <c r="K14" s="20" t="s">
-        <v>40</v>
+      <c r="K14" s="22" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="10" t="n">
+      <c r="A16" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="12" t="n">
         <f aca="false">SUM(I17:I18)</f>
         <v>7403</v>
       </c>
-      <c r="J16" s="11" t="n">
+      <c r="J16" s="13" t="n">
         <f aca="false">IF(OR($I16="",$I$22=0),"",$I16/$I$22)</f>
         <v>0.101100041652726</v>
       </c>
-      <c r="K16" s="9"/>
+      <c r="K16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="B17" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C17" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="D17" s="14"/>
-      <c r="E17" s="15" t="n">
+      <c r="A17" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="16"/>
+      <c r="E17" s="17" t="n">
         <v>50</v>
       </c>
-      <c r="F17" s="16" t="n">
+      <c r="F17" s="18" t="n">
         <v>14</v>
       </c>
-      <c r="G17" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="H17" s="16" t="n">
+      <c r="G17" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="H17" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="I17" s="18" t="n">
-        <f aca="false">IF($E17="","",$E17*$B$6*IF($F17="",1,$F17)*IF($H17="",1,$H17))</f>
+      <c r="I17" s="20" t="n">
+        <f aca="false">IF($E17="","",$E17*$E$6*IF($F17="",1,$F17)*IF($H17="",1,$H17))</f>
         <v>4711</v>
       </c>
-      <c r="J17" s="19" t="n">
+      <c r="J17" s="21" t="n">
         <f aca="false">IF(OR($I17="",$I$22=0),"",$I17/$I$22)</f>
         <v>0.0643363901426435</v>
       </c>
-      <c r="K17" s="20" t="s">
-        <v>46</v>
+      <c r="K17" s="22" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="B18" s="13" t="s">
+      <c r="A18" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="16"/>
+      <c r="E18" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="F18" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="G18" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="D18" s="14"/>
-      <c r="E18" s="15" t="n">
-        <v>50</v>
-      </c>
-      <c r="F18" s="16" t="n">
-        <v>8</v>
-      </c>
-      <c r="G18" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="H18" s="16" t="n">
+      <c r="H18" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="I18" s="18" t="n">
-        <f aca="false">IF($E18="","",$E18*$B$6*IF($F18="",1,$F18)*IF($H18="",1,$H18))</f>
+      <c r="I18" s="20" t="n">
+        <f aca="false">IF($E18="","",$E18*$E$6*IF($F18="",1,$F18)*IF($H18="",1,$H18))</f>
         <v>2692</v>
       </c>
-      <c r="J18" s="19" t="n">
+      <c r="J18" s="21" t="n">
         <f aca="false">IF(OR($I18="",$I$22=0),"",$I18/$I$22)</f>
         <v>0.036763651510082</v>
       </c>
-      <c r="K18" s="20" t="s">
-        <v>49</v>
+      <c r="K18" s="22" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="B20" s="22" t="s">
-        <v>51</v>
-      </c>
-      <c r="C20" s="21"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="23" t="n">
+      <c r="A20" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="25" t="n">
         <v>3000</v>
       </c>
-      <c r="F20" s="21"/>
-      <c r="G20" s="21" t="s">
-        <v>18</v>
-      </c>
-      <c r="H20" s="21"/>
-      <c r="I20" s="24" t="n">
+      <c r="F20" s="23"/>
+      <c r="G20" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="H20" s="23"/>
+      <c r="I20" s="26" t="n">
         <f aca="false">IF($E20="","",$E20*IF($F20="",1,$F20)*IF($H20="",1,$H20))</f>
         <v>3000</v>
       </c>
-      <c r="J20" s="25" t="n">
+      <c r="J20" s="27" t="n">
         <f aca="false">IF(OR($I20="",$I$22=0),"",$I20/$I$22)</f>
         <v>0.0409698939562578</v>
       </c>
-      <c r="K20" s="22"/>
+      <c r="K20" s="24"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="26"/>
-      <c r="B22" s="27" t="s">
-        <v>52</v>
-      </c>
-      <c r="C22" s="26"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="26"/>
-      <c r="F22" s="26"/>
-      <c r="G22" s="26"/>
-      <c r="H22" s="26"/>
-      <c r="I22" s="28" t="n">
+      <c r="A22" s="28"/>
+      <c r="B22" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="C22" s="28"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="28"/>
+      <c r="F22" s="28"/>
+      <c r="G22" s="28"/>
+      <c r="H22" s="28"/>
+      <c r="I22" s="30" t="n">
         <f aca="false">I8+I13+I16+I20</f>
         <v>73224.5</v>
       </c>
-      <c r="J22" s="29" t="n">
+      <c r="J22" s="31" t="n">
         <f aca="false">IF($I$22=0,"",1)</f>
         <v>1</v>
       </c>
-      <c r="K22" s="30"/>
+      <c r="K22" s="32"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Remove project name row from header
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013sgCJY4DwRWjuY7qnd4uaw
</commit_message>
<xml_diff>
--- a/TIFF行程预算.xlsx
+++ b/TIFF行程预算.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="54">
   <si>
     <r>
       <rPr>
@@ -68,30 +68,6 @@
   </si>
   <si>
     <t xml:space="preserve">Beans and Belief</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">项目名称</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="9"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">:</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">TIFF</t>
   </si>
   <si>
     <r>
@@ -985,7 +961,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="32">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1010,11 +986,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1429,387 +1401,383 @@
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="7" t="n">
+      <c r="B6" s="6" t="n">
         <v>6.73</v>
       </c>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="D7" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="E7" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="F7" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="G7" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="H7" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="I7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="J7" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="I7" s="8" t="s">
+      <c r="K7" s="8" t="s">
         <v>21</v>
-      </c>
-      <c r="J7" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="K7" s="9" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="12" t="n">
+      <c r="A8" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="11" t="n">
         <f aca="false">SUM(I9:I11)</f>
         <v>32200</v>
       </c>
-      <c r="J8" s="13" t="n">
+      <c r="J8" s="12" t="n">
         <f aca="false">IF(OR($I8="",$I$22=0),"",$I8/$I$22)</f>
         <v>0.439743528463834</v>
       </c>
-      <c r="K8" s="11"/>
+      <c r="K8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="D9" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="E9" s="16" t="n">
+        <v>2200</v>
+      </c>
+      <c r="F9" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="D9" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="E9" s="17" t="n">
-        <v>2200</v>
-      </c>
-      <c r="F9" s="18" t="n">
+      <c r="H9" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="H9" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="I9" s="20" t="n">
+      <c r="I9" s="19" t="n">
         <f aca="false">IF($E9="","",$E9*IF($F9="",1,$F9)*IF($H9="",1,$H9))</f>
         <v>2200</v>
       </c>
-      <c r="J9" s="21" t="n">
+      <c r="J9" s="20" t="n">
         <f aca="false">IF(OR($I9="",$I$22=0),"",$I9/$I$22)</f>
         <v>0.0300445889012557</v>
       </c>
-      <c r="K9" s="15" t="s">
-        <v>30</v>
+      <c r="K9" s="14" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>18000</v>
+      </c>
+      <c r="F10" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" s="17" t="n">
-        <v>18000</v>
-      </c>
-      <c r="F10" s="18" t="n">
+      <c r="H10" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="H10" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" s="20" t="n">
+      <c r="I10" s="19" t="n">
         <f aca="false">IF($E10="","",$E10*IF($F10="",1,$F10)*IF($H10="",1,$H10))</f>
         <v>18000</v>
       </c>
-      <c r="J10" s="21" t="n">
+      <c r="J10" s="20" t="n">
         <f aca="false">IF(OR($I10="",$I$22=0),"",$I10/$I$22)</f>
         <v>0.245819363737547</v>
       </c>
-      <c r="K10" s="15" t="s">
-        <v>34</v>
+      <c r="K10" s="14" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="B11" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="E11" s="17" t="n">
+      <c r="E11" s="16" t="n">
         <v>12000</v>
       </c>
-      <c r="F11" s="18" t="n">
+      <c r="F11" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="H11" s="18" t="n">
+      <c r="G11" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="H11" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="I11" s="20" t="n">
+      <c r="I11" s="19" t="n">
         <f aca="false">IF($E11="","",$E11*IF($F11="",1,$F11)*IF($H11="",1,$H11))</f>
         <v>12000</v>
       </c>
-      <c r="J11" s="21" t="n">
+      <c r="J11" s="20" t="n">
         <f aca="false">IF(OR($I11="",$I$22=0),"",$I11/$I$22)</f>
         <v>0.163879575825031</v>
       </c>
-      <c r="K11" s="15" t="s">
-        <v>33</v>
+      <c r="K11" s="14" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="12" t="n">
+      <c r="A13" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="11" t="n">
         <f aca="false">SUM(I14:I14)</f>
         <v>30621.5</v>
       </c>
-      <c r="J13" s="13" t="n">
+      <c r="J13" s="12" t="n">
         <f aca="false">IF(OR($I13="",$I$22=0),"",$I13/$I$22)</f>
         <v>0.418186535927183</v>
       </c>
-      <c r="K13" s="11"/>
+      <c r="K13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="14" t="s">
+      <c r="A14" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" s="15"/>
+      <c r="E14" s="16" t="n">
+        <v>350</v>
+      </c>
+      <c r="F14" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="G14" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="C14" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="D14" s="16"/>
-      <c r="E14" s="17" t="n">
-        <v>350</v>
-      </c>
-      <c r="F14" s="18" t="n">
-        <v>13</v>
-      </c>
-      <c r="G14" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="H14" s="18" t="n">
+      <c r="H14" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="I14" s="20" t="n">
-        <f aca="false">IF($E14="","",$E14*$E$6*IF($F14="",1,$F14)*IF($H14="",1,$H14))</f>
+      <c r="I14" s="19" t="n">
+        <f aca="false">IF($E14="","",$E14*$B$6*IF($F14="",1,$F14)*IF($H14="",1,$H14))</f>
         <v>30621.5</v>
       </c>
-      <c r="J14" s="21" t="n">
+      <c r="J14" s="20" t="n">
         <f aca="false">IF(OR($I14="",$I$22=0),"",$I14/$I$22)</f>
         <v>0.418186535927183</v>
       </c>
-      <c r="K14" s="22" t="s">
-        <v>43</v>
+      <c r="K14" s="21" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="12" t="n">
+      <c r="A16" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="11" t="n">
         <f aca="false">SUM(I17:I18)</f>
         <v>7403</v>
       </c>
-      <c r="J16" s="13" t="n">
+      <c r="J16" s="12" t="n">
         <f aca="false">IF(OR($I16="",$I$22=0),"",$I16/$I$22)</f>
         <v>0.101100041652726</v>
       </c>
-      <c r="K16" s="11"/>
+      <c r="K16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="D17" s="15"/>
+      <c r="E17" s="16" t="n">
+        <v>50</v>
+      </c>
+      <c r="F17" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="G17" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="B17" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="C17" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="D17" s="16"/>
-      <c r="E17" s="17" t="n">
-        <v>50</v>
-      </c>
-      <c r="F17" s="18" t="n">
-        <v>14</v>
-      </c>
-      <c r="G17" s="18" t="s">
-        <v>48</v>
-      </c>
-      <c r="H17" s="18" t="n">
+      <c r="H17" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="I17" s="20" t="n">
-        <f aca="false">IF($E17="","",$E17*$E$6*IF($F17="",1,$F17)*IF($H17="",1,$H17))</f>
+      <c r="I17" s="19" t="n">
+        <f aca="false">IF($E17="","",$E17*$B$6*IF($F17="",1,$F17)*IF($H17="",1,$H17))</f>
         <v>4711</v>
       </c>
-      <c r="J17" s="21" t="n">
+      <c r="J17" s="20" t="n">
         <f aca="false">IF(OR($I17="",$I$22=0),"",$I17/$I$22)</f>
         <v>0.0643363901426435</v>
       </c>
-      <c r="K17" s="22" t="s">
-        <v>49</v>
+      <c r="K17" s="21" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
+      <c r="A18" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="D18" s="15"/>
+      <c r="E18" s="16" t="n">
         <v>50</v>
       </c>
-      <c r="B18" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="C18" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="D18" s="16"/>
-      <c r="E18" s="17" t="n">
-        <v>50</v>
-      </c>
-      <c r="F18" s="18" t="n">
+      <c r="F18" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="G18" s="18" t="s">
-        <v>48</v>
-      </c>
-      <c r="H18" s="18" t="n">
+      <c r="G18" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="H18" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="I18" s="20" t="n">
-        <f aca="false">IF($E18="","",$E18*$E$6*IF($F18="",1,$F18)*IF($H18="",1,$H18))</f>
+      <c r="I18" s="19" t="n">
+        <f aca="false">IF($E18="","",$E18*$B$6*IF($F18="",1,$F18)*IF($H18="",1,$H18))</f>
         <v>2692</v>
       </c>
-      <c r="J18" s="21" t="n">
+      <c r="J18" s="20" t="n">
         <f aca="false">IF(OR($I18="",$I$22=0),"",$I18/$I$22)</f>
         <v>0.036763651510082</v>
       </c>
-      <c r="K18" s="22" t="s">
-        <v>52</v>
+      <c r="K18" s="21" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="23" t="s">
-        <v>53</v>
-      </c>
-      <c r="B20" s="24" t="s">
-        <v>54</v>
-      </c>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="25" t="n">
+      <c r="A20" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" s="23" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="24" t="n">
         <v>3000</v>
       </c>
-      <c r="F20" s="23"/>
-      <c r="G20" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="H20" s="23"/>
-      <c r="I20" s="26" t="n">
+      <c r="F20" s="22"/>
+      <c r="G20" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="H20" s="22"/>
+      <c r="I20" s="25" t="n">
         <f aca="false">IF($E20="","",$E20*IF($F20="",1,$F20)*IF($H20="",1,$H20))</f>
         <v>3000</v>
       </c>
-      <c r="J20" s="27" t="n">
+      <c r="J20" s="26" t="n">
         <f aca="false">IF(OR($I20="",$I$22=0),"",$I20/$I$22)</f>
         <v>0.0409698939562578</v>
       </c>
-      <c r="K20" s="24"/>
+      <c r="K20" s="23"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="28"/>
-      <c r="B22" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="C22" s="28"/>
-      <c r="D22" s="28"/>
-      <c r="E22" s="28"/>
-      <c r="F22" s="28"/>
-      <c r="G22" s="28"/>
-      <c r="H22" s="28"/>
-      <c r="I22" s="30" t="n">
+      <c r="A22" s="27"/>
+      <c r="B22" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="C22" s="27"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="27"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="27"/>
+      <c r="I22" s="29" t="n">
         <f aca="false">I8+I13+I16+I20</f>
         <v>73224.5</v>
       </c>
-      <c r="J22" s="31" t="n">
+      <c r="J22" s="30" t="n">
         <f aca="false">IF($I$22=0,"",1)</f>
         <v>1</v>
       </c>
-      <c r="K22" s="32"/>
+      <c r="K22" s="31"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>